<commit_message>
CAMBIOS DE FONDO LOGIN
</commit_message>
<xml_diff>
--- a/Datos.xlsx
+++ b/Datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chanitosfrutas-my.sharepoint.com/personal/bescobedo_chanitos_com/Documents/WorkSpace/preenfrio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="13_ncr:1_{F0A36C04-E6E5-4B51-9906-23526A19135B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E3B267F-3F95-4AD3-B07C-FE818ADA9922}"/>
+  <xr:revisionPtr revIDLastSave="312" documentId="13_ncr:1_{F0A36C04-E6E5-4B51-9906-23526A19135B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93BDAFDF-E20C-4591-9833-435D6350C2B7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{870F0A8F-B5CF-4FD7-9FD6-C646EB212759}"/>
+    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{870F0A8F-B5CF-4FD7-9FD6-C646EB212759}"/>
   </bookViews>
   <sheets>
     <sheet name="PREENFRIO" sheetId="1" r:id="rId1"/>
@@ -6241,7 +6241,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E6D9E-686A-4183-92BF-9B0AF16F6985}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R284"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6300,7 +6299,7 @@
         <v>1119</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>131</v>
       </c>
@@ -6349,7 +6348,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>115</v>
       </c>
@@ -6399,7 +6398,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>106</v>
       </c>
@@ -6449,7 +6448,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>123</v>
       </c>
@@ -6499,7 +6498,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>534</v>
       </c>
@@ -6549,7 +6548,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>532</v>
       </c>
@@ -6599,7 +6598,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>557</v>
       </c>
@@ -6649,7 +6648,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>117</v>
       </c>
@@ -6699,7 +6698,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>98</v>
       </c>
@@ -6749,7 +6748,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>146</v>
       </c>
@@ -6799,7 +6798,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>144</v>
       </c>
@@ -6849,7 +6848,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>127</v>
       </c>
@@ -6899,7 +6898,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>479</v>
       </c>
@@ -6949,7 +6948,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>137</v>
       </c>
@@ -6999,7 +6998,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>139</v>
       </c>
@@ -7049,7 +7048,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>141</v>
       </c>
@@ -7099,7 +7098,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>110</v>
       </c>
@@ -7149,7 +7148,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>475</v>
       </c>
@@ -7199,7 +7198,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>481</v>
       </c>
@@ -7249,7 +7248,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>516</v>
       </c>
@@ -7299,7 +7298,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>559</v>
       </c>
@@ -7349,7 +7348,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>133</v>
       </c>
@@ -7399,7 +7398,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>142</v>
       </c>
@@ -7449,7 +7448,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>96</v>
       </c>
@@ -7499,7 +7498,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>100</v>
       </c>
@@ -7549,7 +7548,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>555</v>
       </c>
@@ -7599,7 +7598,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>418</v>
       </c>
@@ -7649,7 +7648,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>104</v>
       </c>
@@ -7699,7 +7698,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>148</v>
       </c>
@@ -7749,7 +7748,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>102</v>
       </c>
@@ -7799,7 +7798,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>108</v>
       </c>
@@ -7849,7 +7848,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>530</v>
       </c>
@@ -7899,7 +7898,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>135</v>
       </c>
@@ -7949,7 +7948,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>129</v>
       </c>
@@ -7999,7 +7998,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>121</v>
       </c>
@@ -8049,7 +8048,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>119</v>
       </c>
@@ -8099,7 +8098,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>125</v>
       </c>
@@ -8149,7 +8148,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>114</v>
       </c>
@@ -8199,7 +8198,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>112</v>
       </c>
@@ -8249,7 +8248,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>477</v>
       </c>
@@ -8299,7 +8298,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>536</v>
       </c>
@@ -8349,7 +8348,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>392</v>
       </c>
@@ -8399,7 +8398,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>198</v>
       </c>
@@ -8449,7 +8448,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>163</v>
       </c>
@@ -8499,7 +8498,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>261</v>
       </c>
@@ -8549,7 +8548,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>153</v>
       </c>
@@ -8599,7 +8598,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>430</v>
       </c>
@@ -8649,7 +8648,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>170</v>
       </c>
@@ -8699,7 +8698,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>368</v>
       </c>
@@ -8749,7 +8748,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>565</v>
       </c>
@@ -8799,7 +8798,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>308</v>
       </c>
@@ -8849,7 +8848,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>400</v>
       </c>
@@ -8899,7 +8898,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>226</v>
       </c>
@@ -8949,7 +8948,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>225</v>
       </c>
@@ -8999,7 +8998,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>328</v>
       </c>
@@ -9049,7 +9048,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
         <v>432</v>
       </c>
@@ -9099,7 +9098,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
         <v>188</v>
       </c>
@@ -9149,7 +9148,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>561</v>
       </c>
@@ -9199,7 +9198,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
         <v>189</v>
       </c>
@@ -9249,7 +9248,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
         <v>343</v>
       </c>
@@ -9299,7 +9298,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>318</v>
       </c>
@@ -9349,7 +9348,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>330</v>
       </c>
@@ -9399,7 +9398,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>168</v>
       </c>
@@ -9449,7 +9448,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>172</v>
       </c>
@@ -9499,7 +9498,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>242</v>
       </c>
@@ -9549,7 +9548,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>287</v>
       </c>
@@ -9599,7 +9598,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>366</v>
       </c>
@@ -9649,7 +9648,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>567</v>
       </c>
@@ -9699,7 +9698,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>233</v>
       </c>
@@ -9749,7 +9748,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>484</v>
       </c>
@@ -9799,7 +9798,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
         <v>251</v>
       </c>
@@ -9849,7 +9848,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>391</v>
       </c>
@@ -9899,7 +9898,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>553</v>
       </c>
@@ -9949,7 +9948,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>150</v>
       </c>
@@ -9999,7 +9998,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>196</v>
       </c>
@@ -10049,7 +10048,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>364</v>
       </c>
@@ -10099,7 +10098,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>365</v>
       </c>
@@ -10149,7 +10148,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>398</v>
       </c>
@@ -10199,7 +10198,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>538</v>
       </c>
@@ -10249,7 +10248,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>267</v>
       </c>
@@ -10299,7 +10298,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>200</v>
       </c>
@@ -10349,7 +10348,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>346</v>
       </c>
@@ -10399,7 +10398,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>352</v>
       </c>
@@ -10449,7 +10448,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>355</v>
       </c>
@@ -10499,7 +10498,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>212</v>
       </c>
@@ -10549,7 +10548,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>442</v>
       </c>
@@ -10599,7 +10598,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>449</v>
       </c>
@@ -10649,7 +10648,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>275</v>
       </c>
@@ -10699,7 +10698,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>349</v>
       </c>
@@ -10749,7 +10748,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>273</v>
       </c>
@@ -10799,7 +10798,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>428</v>
       </c>
@@ -10849,7 +10848,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>177</v>
       </c>
@@ -10899,7 +10898,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>205</v>
       </c>
@@ -10949,7 +10948,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>446</v>
       </c>
@@ -10999,7 +10998,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>486</v>
       </c>
@@ -11049,7 +11048,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>455</v>
       </c>
@@ -11099,7 +11098,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>310</v>
       </c>
@@ -11149,7 +11148,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>537</v>
       </c>
@@ -11199,7 +11198,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A100" s="6" t="s">
         <v>407</v>
       </c>
@@ -11249,7 +11248,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>203</v>
       </c>
@@ -11299,7 +11298,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
         <v>219</v>
       </c>
@@ -11349,7 +11348,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
         <v>437</v>
       </c>
@@ -11399,7 +11398,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A104" s="6" t="s">
         <v>509</v>
       </c>
@@ -11449,7 +11448,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
         <v>238</v>
       </c>
@@ -11499,7 +11498,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
         <v>569</v>
       </c>
@@ -11549,7 +11548,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
         <v>320</v>
       </c>
@@ -11599,7 +11598,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A108" s="6" t="s">
         <v>572</v>
       </c>
@@ -11649,7 +11648,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
         <v>340</v>
       </c>
@@ -11699,7 +11698,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A110" s="6" t="s">
         <v>295</v>
       </c>
@@ -11749,7 +11748,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A111" s="6" t="s">
         <v>459</v>
       </c>
@@ -11799,7 +11798,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A112" s="6" t="s">
         <v>290</v>
       </c>
@@ -11849,7 +11848,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A113" s="6" t="s">
         <v>305</v>
       </c>
@@ -11899,7 +11898,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A114" s="6" t="s">
         <v>324</v>
       </c>
@@ -11949,7 +11948,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A115" s="6" t="s">
         <v>271</v>
       </c>
@@ -11999,7 +11998,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A116" s="6" t="s">
         <v>316</v>
       </c>
@@ -12049,7 +12048,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A117" s="6" t="s">
         <v>374</v>
       </c>
@@ -12099,7 +12098,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A118" s="6" t="s">
         <v>376</v>
       </c>
@@ -12149,7 +12148,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
         <v>436</v>
       </c>
@@ -12199,7 +12198,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A120" s="6" t="s">
         <v>217</v>
       </c>
@@ -12249,7 +12248,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A121" s="6" t="s">
         <v>307</v>
       </c>
@@ -12299,7 +12298,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
         <v>568</v>
       </c>
@@ -12349,7 +12348,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
         <v>506</v>
       </c>
@@ -12399,7 +12398,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A124" s="6" t="s">
         <v>231</v>
       </c>
@@ -12449,7 +12448,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A125" s="6" t="s">
         <v>159</v>
       </c>
@@ -12499,7 +12498,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
         <v>548</v>
       </c>
@@ -12549,7 +12548,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>161</v>
       </c>
@@ -12599,7 +12598,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A128" s="6" t="s">
         <v>422</v>
       </c>
@@ -12649,7 +12648,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>491</v>
       </c>
@@ -12699,7 +12698,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>494</v>
       </c>
@@ -12749,7 +12748,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
         <v>298</v>
       </c>
@@ -12799,7 +12798,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A132" s="6" t="s">
         <v>288</v>
       </c>
@@ -12849,7 +12848,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A133" s="6" t="s">
         <v>405</v>
       </c>
@@ -12899,7 +12898,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
         <v>383</v>
       </c>
@@ -12949,7 +12948,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A135" s="6" t="s">
         <v>245</v>
       </c>
@@ -12999,7 +12998,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A136" s="6" t="s">
         <v>372</v>
       </c>
@@ -13049,7 +13048,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A137" s="6" t="s">
         <v>502</v>
       </c>
@@ -13099,7 +13098,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A138" s="6" t="s">
         <v>541</v>
       </c>
@@ -13149,7 +13148,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>381</v>
       </c>
@@ -13199,7 +13198,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A140" s="6" t="s">
         <v>247</v>
       </c>
@@ -13249,7 +13248,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A141" s="6" t="s">
         <v>439</v>
       </c>
@@ -13299,7 +13298,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
         <v>357</v>
       </c>
@@ -13349,7 +13348,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A143" s="6" t="s">
         <v>157</v>
       </c>
@@ -13399,7 +13398,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>332</v>
       </c>
@@ -13449,7 +13448,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A145" s="6" t="s">
         <v>279</v>
       </c>
@@ -13499,7 +13498,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A146" s="6" t="s">
         <v>263</v>
       </c>
@@ -13549,7 +13548,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A147" s="6" t="s">
         <v>496</v>
       </c>
@@ -13599,7 +13598,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A148" s="6" t="s">
         <v>249</v>
       </c>
@@ -13649,7 +13648,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="149" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
         <v>379</v>
       </c>
@@ -13699,7 +13698,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A150" s="6" t="s">
         <v>377</v>
       </c>
@@ -13749,7 +13748,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A151" s="6" t="s">
         <v>370</v>
       </c>
@@ -13799,7 +13798,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="152" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A152" s="6" t="s">
         <v>155</v>
       </c>
@@ -14599,7 +14598,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="168" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A168" s="6" t="s">
         <v>394</v>
       </c>
@@ -14649,7 +14648,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="169" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A169" s="6" t="s">
         <v>444</v>
       </c>
@@ -14699,7 +14698,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="170" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A170" s="6" t="s">
         <v>326</v>
       </c>
@@ -14749,7 +14748,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="171" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A171" s="6" t="s">
         <v>359</v>
       </c>
@@ -14799,7 +14798,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="172" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A172" s="6" t="s">
         <v>302</v>
       </c>
@@ -14849,7 +14848,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="173" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A173" s="6" t="s">
         <v>519</v>
       </c>
@@ -14899,7 +14898,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="174" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
         <v>322</v>
       </c>
@@ -14949,7 +14948,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="175" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A175" s="6" t="s">
         <v>411</v>
       </c>
@@ -14999,7 +14998,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>296</v>
       </c>
@@ -15049,7 +15048,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="177" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>214</v>
       </c>
@@ -15099,7 +15098,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="178" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>216</v>
       </c>
@@ -15149,7 +15148,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="179" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>483</v>
       </c>
@@ -15199,7 +15198,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="180" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A180" s="6" t="s">
         <v>210</v>
       </c>
@@ -15249,7 +15248,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="181" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
         <v>363</v>
       </c>
@@ -15299,7 +15298,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="182" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
         <v>453</v>
       </c>
@@ -15349,7 +15348,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="183" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
         <v>253</v>
       </c>
@@ -15399,7 +15398,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="184" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A184" s="6" t="s">
         <v>414</v>
       </c>
@@ -15449,7 +15448,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A185" s="6" t="s">
         <v>283</v>
       </c>
@@ -15499,7 +15498,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A186" s="6" t="s">
         <v>221</v>
       </c>
@@ -15549,7 +15548,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="187" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A187" s="6" t="s">
         <v>424</v>
       </c>
@@ -15599,7 +15598,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="188" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A188" s="6" t="s">
         <v>181</v>
       </c>
@@ -15649,7 +15648,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="189" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A189" s="6" t="s">
         <v>426</v>
       </c>
@@ -15699,7 +15698,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="190" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A190" s="6" t="s">
         <v>416</v>
       </c>
@@ -15749,7 +15748,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A191" s="6" t="s">
         <v>194</v>
       </c>
@@ -15799,7 +15798,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A192" s="6" t="s">
         <v>312</v>
       </c>
@@ -15849,7 +15848,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="193" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A193" s="6" t="s">
         <v>183</v>
       </c>
@@ -15899,7 +15898,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="194" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A194" s="6" t="s">
         <v>185</v>
       </c>
@@ -15949,7 +15948,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A195" s="6" t="s">
         <v>336</v>
       </c>
@@ -15999,7 +15998,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A196" s="6" t="s">
         <v>281</v>
       </c>
@@ -16049,7 +16048,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A197" s="6" t="s">
         <v>338</v>
       </c>
@@ -16099,7 +16098,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A198" s="6" t="s">
         <v>334</v>
       </c>
@@ -16149,7 +16148,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A199" s="6" t="s">
         <v>434</v>
       </c>
@@ -16199,7 +16198,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A200" s="6" t="s">
         <v>419</v>
       </c>
@@ -16249,7 +16248,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A201" s="6" t="s">
         <v>513</v>
       </c>
@@ -16299,7 +16298,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A202" s="6" t="s">
         <v>269</v>
       </c>
@@ -16349,7 +16348,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="203" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A203" s="6" t="s">
         <v>462</v>
       </c>
@@ -16399,7 +16398,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A204" s="6" t="s">
         <v>174</v>
       </c>
@@ -16449,7 +16448,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="205" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A205" s="6" t="s">
         <v>385</v>
       </c>
@@ -16499,7 +16498,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="206" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A206" s="6" t="s">
         <v>460</v>
       </c>
@@ -16549,7 +16548,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="207" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A207" s="6" t="s">
         <v>176</v>
       </c>
@@ -16599,7 +16598,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="208" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A208" s="6" t="s">
         <v>539</v>
       </c>
@@ -16649,7 +16648,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="209" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A209" s="6" t="s">
         <v>653</v>
       </c>
@@ -16699,7 +16698,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="210" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A210" s="6" t="s">
         <v>165</v>
       </c>
@@ -16749,7 +16748,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="211" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A211" s="6" t="s">
         <v>311</v>
       </c>
@@ -16799,7 +16798,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="212" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A212" s="6" t="s">
         <v>348</v>
       </c>
@@ -16849,7 +16848,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A213" s="6" t="s">
         <v>285</v>
       </c>
@@ -16899,7 +16898,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="214" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A214" s="6" t="s">
         <v>228</v>
       </c>
@@ -16949,7 +16948,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="215" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A215" s="6" t="s">
         <v>493</v>
       </c>
@@ -16999,7 +16998,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="216" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A216" s="6" t="s">
         <v>230</v>
       </c>
@@ -17049,7 +17048,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="217" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A217" s="6" t="s">
         <v>227</v>
       </c>
@@ -17099,7 +17098,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="218" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A218" s="6" t="s">
         <v>223</v>
       </c>
@@ -17149,7 +17148,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="219" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A219" s="6" t="s">
         <v>229</v>
       </c>
@@ -17199,7 +17198,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="220" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A220" s="6" t="s">
         <v>341</v>
       </c>
@@ -17249,7 +17248,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="221" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A221" s="6" t="s">
         <v>292</v>
       </c>
@@ -17299,7 +17298,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="222" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A222" s="6" t="s">
         <v>294</v>
       </c>
@@ -17349,7 +17348,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="223" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A223" s="6" t="s">
         <v>457</v>
       </c>
@@ -17399,7 +17398,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="224" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A224" s="6" t="s">
         <v>300</v>
       </c>
@@ -17449,7 +17448,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="225" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A225" s="6" t="s">
         <v>240</v>
       </c>
@@ -17499,7 +17498,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="226" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A226" s="6" t="s">
         <v>518</v>
       </c>
@@ -17549,7 +17548,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="227" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A227" s="6" t="s">
         <v>409</v>
       </c>
@@ -17599,7 +17598,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="228" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A228" s="6" t="s">
         <v>235</v>
       </c>
@@ -17649,7 +17648,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="229" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A229" s="6" t="s">
         <v>539</v>
       </c>
@@ -17699,7 +17698,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="230" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A230" s="6" t="s">
         <v>243</v>
       </c>
@@ -17749,7 +17748,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="231" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A231" s="6" t="s">
         <v>265</v>
       </c>
@@ -17799,7 +17798,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="232" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A232" s="6" t="s">
         <v>540</v>
       </c>
@@ -17849,7 +17848,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="233" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A233" s="6" t="s">
         <v>152</v>
       </c>
@@ -17899,7 +17898,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="234" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A234" s="6" t="s">
         <v>387</v>
       </c>
@@ -17949,7 +17948,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="235" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A235" s="6" t="s">
         <v>344</v>
       </c>
@@ -17999,7 +17998,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="236" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A236" s="6" t="s">
         <v>361</v>
       </c>
@@ -18049,7 +18048,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="237" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A237" s="6" t="s">
         <v>402</v>
       </c>
@@ -18099,7 +18098,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="238" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A238" s="6" t="s">
         <v>404</v>
       </c>
@@ -18149,7 +18148,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="239" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A239" s="6" t="s">
         <v>314</v>
       </c>
@@ -18199,7 +18198,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="240" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A240" s="6" t="s">
         <v>255</v>
       </c>
@@ -18249,7 +18248,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="241" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A241" s="6" t="s">
         <v>396</v>
       </c>
@@ -18299,7 +18298,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="242" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A242" s="6" t="s">
         <v>191</v>
       </c>
@@ -18349,7 +18348,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="243" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A243" s="6" t="s">
         <v>179</v>
       </c>
@@ -18399,7 +18398,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="244" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A244" s="6" t="s">
         <v>236</v>
       </c>
@@ -18449,7 +18448,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="245" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A245" s="6" t="s">
         <v>208</v>
       </c>
@@ -18499,7 +18498,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="246" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A246" s="6" t="s">
         <v>166</v>
       </c>
@@ -18549,7 +18548,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="247" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A247" s="6" t="s">
         <v>500</v>
       </c>
@@ -18599,7 +18598,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="248" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A248" s="6" t="s">
         <v>545</v>
       </c>
@@ -18649,7 +18648,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="249" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A249" s="6" t="s">
         <v>546</v>
       </c>
@@ -18699,7 +18698,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="250" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A250" s="6" t="s">
         <v>202</v>
       </c>
@@ -18749,7 +18748,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="251" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A251" s="6" t="s">
         <v>499</v>
       </c>
@@ -18799,7 +18798,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="252" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A252" s="6" t="s">
         <v>489</v>
       </c>
@@ -18849,7 +18848,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="253" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A253" s="6" t="s">
         <v>490</v>
       </c>
@@ -18899,7 +18898,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="254" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A254" s="6" t="s">
         <v>354</v>
       </c>
@@ -18949,7 +18948,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="255" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A255" s="6" t="s">
         <v>448</v>
       </c>
@@ -18999,7 +18998,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="256" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A256" s="6" t="s">
         <v>447</v>
       </c>
@@ -19049,7 +19048,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="257" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A257" s="6" t="s">
         <v>452</v>
       </c>
@@ -19099,7 +19098,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="258" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A258" s="6" t="s">
         <v>451</v>
       </c>
@@ -19149,7 +19148,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A259" s="6" t="s">
         <v>277</v>
       </c>
@@ -19199,7 +19198,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="260" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A260" s="6" t="s">
         <v>278</v>
       </c>
@@ -19249,7 +19248,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="261" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A261" s="6" t="s">
         <v>351</v>
       </c>
@@ -19299,7 +19298,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="262" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A262" s="6" t="s">
         <v>207</v>
       </c>
@@ -19349,7 +19348,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="263" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A263" s="6" t="s">
         <v>564</v>
       </c>
@@ -19399,7 +19398,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="264" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A264" s="6" t="s">
         <v>511</v>
       </c>
@@ -19449,7 +19448,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="265" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A265" s="6" t="s">
         <v>549</v>
       </c>
@@ -19499,7 +19498,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="266" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A266" s="6" t="s">
         <v>445</v>
       </c>
@@ -19549,7 +19548,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="267" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A267" s="6" t="s">
         <v>193</v>
       </c>
@@ -19599,7 +19598,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="268" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A268" s="6" t="s">
         <v>508</v>
       </c>
@@ -19649,7 +19648,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A269" s="6" t="s">
         <v>488</v>
       </c>
@@ -19699,7 +19698,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="270" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A270" s="6" t="s">
         <v>469</v>
       </c>
@@ -19749,7 +19748,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="271" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A271" s="6" t="s">
         <v>471</v>
       </c>
@@ -19799,7 +19798,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="272" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A272" s="6" t="s">
         <v>526</v>
       </c>
@@ -19849,7 +19848,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="273" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A273" s="6" t="s">
         <v>463</v>
       </c>
@@ -19899,7 +19898,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="274" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A274" s="6" t="s">
         <v>473</v>
       </c>
@@ -19949,7 +19948,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="275" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A275" s="6" t="s">
         <v>543</v>
       </c>
@@ -19999,7 +19998,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="276" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A276" s="6" t="s">
         <v>528</v>
       </c>
@@ -20049,7 +20048,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="277" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A277" s="6" t="s">
         <v>497</v>
       </c>
@@ -20099,7 +20098,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="278" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A278" s="6" t="s">
         <v>465</v>
       </c>
@@ -20149,7 +20148,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="279" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A279" s="6" t="s">
         <v>522</v>
       </c>
@@ -20199,7 +20198,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="280" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A280" s="6" t="s">
         <v>520</v>
       </c>
@@ -20249,7 +20248,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="281" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A281" s="6" t="s">
         <v>571</v>
       </c>
@@ -20299,7 +20298,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="282" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A282" s="6" t="s">
         <v>467</v>
       </c>
@@ -20349,7 +20348,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="283" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A283" s="6" t="s">
         <v>524</v>
       </c>
@@ -20399,7 +20398,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="284" spans="1:18" ht="22.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:18" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A284" s="6" t="s">
         <v>514</v>
       </c>
@@ -20484,13 +20483,7 @@
     <protectedRange algorithmName="SHA-512" hashValue="oAofLzPsEABz+g8s4EYjUuwXH7ykbMbBHfCBkrjaG9AypkvLlHymmath48lOXQru/nByDYQVi/KXn1fge9PtNA==" saltValue="K19iw11Oiq05wm1mPIKVDQ==" spinCount="100000" sqref="D276" name="Rango4_30"/>
     <protectedRange algorithmName="SHA-512" hashValue="oAofLzPsEABz+g8s4EYjUuwXH7ykbMbBHfCBkrjaG9AypkvLlHymmath48lOXQru/nByDYQVi/KXn1fge9PtNA==" saltValue="K19iw11Oiq05wm1mPIKVDQ==" spinCount="100000" sqref="D277" name="Rango4_31"/>
   </protectedRanges>
-  <autoFilter ref="A1:O284" xr:uid="{329E6D9E-686A-4183-92BF-9B0AF16F6985}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="124"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:O284" xr:uid="{329E6D9E-686A-4183-92BF-9B0AF16F6985}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -21849,11 +21842,11 @@
     </row>
   </sheetData>
   <autoFilter ref="B1:D1" xr:uid="{961DD99E-A2C7-4E25-8FB0-84DFB4FA4937}"/>
+  <conditionalFormatting sqref="A1:A39">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A39">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -36458,7 +36451,7 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>